<commit_message>
se ajustaron datos para ficha de riesgo
</commit_message>
<xml_diff>
--- a/backend/src/assets/official_forms/riesgo_oficial.xlsx
+++ b/backend/src/assets/official_forms/riesgo_oficial.xlsx
@@ -1401,8 +1401,10 @@
       <c r="L12" s="15"/>
       <c r="M12" s="15"/>
       <c r="N12" s="26"/>
-      <c r="O12" s="15" t="s">
-        <v>70</v>
+      <c r="O12" s="15" t="inlineStr">
+        <is>
+          <t>Universidad</t>
+        </is>
       </c>
       <c r="P12" s="15"/>
       <c r="Q12" s="15"/>

</xml_diff>

<commit_message>
se ajusto el xlsx de ficha de riesgo
</commit_message>
<xml_diff>
--- a/backend/src/assets/official_forms/riesgo_oficial.xlsx
+++ b/backend/src/assets/official_forms/riesgo_oficial.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Huguito\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\cap_prenatal\backend\src\assets\official_forms\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8487F69A-339E-43F7-815E-C39137A28289}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D154F49A-74A6-4A66-B2E5-833EEB314976}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-23148" yWindow="516" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ficha de riesgo" sheetId="2" r:id="rId1"/>
@@ -232,9 +232,6 @@
     <t xml:space="preserve">  Ninguna:</t>
   </si>
   <si>
-    <t xml:space="preserve"> </t>
-  </si>
-  <si>
     <t xml:space="preserve">   Diversificado</t>
   </si>
   <si>
@@ -248,6 +245,9 @@
   </si>
   <si>
     <t xml:space="preserve">DIRECCION DEPARTAMENTAL DE REDES INTEGRADAS DE SERVICIOS DE SALUD DE PETEN, AREA SUR ORIENTE, UNIDAD DE SALUD REPRODUCTIVA. </t>
+  </si>
+  <si>
+    <t>Universidad</t>
   </si>
 </sst>
 </file>
@@ -342,7 +342,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="12">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -473,11 +473,20 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -518,6 +527,15 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -565,8 +583,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="180976" y="0"/>
-          <a:ext cx="1343024" cy="381000"/>
+          <a:off x="182881" y="0"/>
+          <a:ext cx="1356359" cy="381000"/>
           <a:chOff x="9880271" y="390341"/>
           <a:chExt cx="1981200" cy="892193"/>
         </a:xfrm>
@@ -757,7 +775,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>31</xdr:col>
-      <xdr:colOff>47625</xdr:colOff>
+      <xdr:colOff>41910</xdr:colOff>
       <xdr:row>5</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
@@ -1103,7 +1121,7 @@
   <sheetData>
     <row r="3" spans="2:28" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C3" s="30" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D3" s="30"/>
       <c r="E3" s="30"/>
@@ -1323,7 +1341,7 @@
       <c r="H10" s="15"/>
       <c r="I10" s="26"/>
       <c r="J10" s="15" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="K10" s="15"/>
       <c r="L10" s="26"/>
@@ -1386,7 +1404,7 @@
       <c r="C12" s="15"/>
       <c r="D12" s="15"/>
       <c r="E12" s="15" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="F12" s="15"/>
       <c r="G12" s="26"/>
@@ -1396,18 +1414,16 @@
       <c r="I12" s="15"/>
       <c r="J12" s="26"/>
       <c r="K12" s="15" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="L12" s="15"/>
       <c r="M12" s="15"/>
       <c r="N12" s="26"/>
-      <c r="O12" s="15" t="inlineStr">
-        <is>
-          <t>Universidad</t>
-        </is>
-      </c>
-      <c r="P12" s="15"/>
-      <c r="Q12" s="15"/>
+      <c r="O12" s="33" t="s">
+        <v>75</v>
+      </c>
+      <c r="P12" s="32"/>
+      <c r="Q12" s="34"/>
       <c r="R12" s="26"/>
       <c r="S12" s="15" t="s">
         <v>69</v>
@@ -3004,7 +3020,7 @@
     </row>
     <row r="62" spans="2:29" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B62" s="18" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C62" s="18"/>
       <c r="D62" s="18"/>
@@ -4283,11 +4299,12 @@
       <c r="AB105" s="3"/>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="5">
     <mergeCell ref="B22:R22"/>
     <mergeCell ref="G6:L6"/>
     <mergeCell ref="C3:Y4"/>
     <mergeCell ref="G5:W5"/>
+    <mergeCell ref="O12:Q12"/>
   </mergeCells>
   <printOptions verticalCentered="1"/>
   <pageMargins left="0.31496062992125984" right="0" top="0.15748031496062992" bottom="0.15748031496062992" header="0.31496062992125984" footer="0.31496062992125984"/>

</xml_diff>